<commit_message>
Agregar casco de seguridad (EPP) y lista de subcategorías en el Excel
- Nuevo producto TRU-CAS-001 con foto
- Lista desplegable de Subcategoría y categoría "Protección colectiva"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Productos_Herramientas.xlsx
+++ b/Catalogo_Productos_Herramientas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leo-n\Desktop\Claude Proyectos\1. Tienda Herramientas Online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0988E546-7B39-486B-A06D-545F9FA57CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458024BD-ED82-494C-AA55-E56EEA7FE0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="174">
   <si>
     <t>CÓMO USAR ESTA PLANTILLA</t>
   </si>
@@ -78,9 +78,6 @@
     <t>2. Las filas 4 a 6 son ejemplos con precios inventados: reemplázalas con tus datos reales.</t>
   </si>
   <si>
-    <t>3. Marca, Categoría, Unidad, Garantía, Destacado y Activo se eligen de una lista desplegable.</t>
-  </si>
-  <si>
     <t>4. Las columnas verdes (Precio final, Margen, Estado stock) se calculan solas.</t>
   </si>
   <si>
@@ -376,6 +373,233 @@
   </si>
   <si>
     <t>ALU8D15</t>
+  </si>
+  <si>
+    <t>Descripción larga</t>
+  </si>
+  <si>
+    <t>Taladro percutor de 650 W ideal para perforar concreto, ladrillo, madera y metal. Su función de percusión facilita el trabajo en superficies duras, y el giro reversible permite atornillar y destornillar con comodidad.
+Tiene mandril de 1/2" para brocas de distintos tamaños y velocidad variable de 0 a 3000 rpm para controlar cada perforación. Perfecto para instalaciones, remodelaciones y mantenimiento en casa, taller u obra.
+Recomendación: usa lentes de protección y guantes durante el trabajo.</t>
+  </si>
+  <si>
+    <t>Amoladora angular de 750 W para cortar y desbastar metal, concreto, cerámica y piedra con discos de 4 1/2" (115 mm). Su motor de 11 000 rpm ofrece cortes rápidos y precisos.
+Cuenta con mango lateral para un mejor control y guarda de protección. Ideal para metalmecánica, construcción y mantenimiento.
+Recomendación: usa siempre lentes o careta de protección, guantes y el disco adecuado para cada material.</t>
+  </si>
+  <si>
+    <t>Alicate universal de 8" fabricado en acero alto carbono, con cuerpo forjado y filos endurecidos para cortar, sujetar, doblar y torcer alambres y cables.
+Sus mangos ergonómicos de PVC bicolor brindan un agarre firme y cómodo durante el uso prolongado. Una herramienta básica para electricistas, mecánicos, técnicos y el hogar.
+Importante: el mango no está aislado; no lo uses en circuitos con corriente eléctrica.</t>
+  </si>
+  <si>
+    <t>TRU-CAS-001</t>
+  </si>
+  <si>
+    <t>Casco de seguridad con ratchet blanco</t>
+  </si>
+  <si>
+    <t>Cascos</t>
+  </si>
+  <si>
+    <t>Rotomartillos</t>
+  </si>
+  <si>
+    <t>Atornilladores</t>
+  </si>
+  <si>
+    <t>Lijadoras</t>
+  </si>
+  <si>
+    <t>Pistolas de calor</t>
+  </si>
+  <si>
+    <t>Soldadoras</t>
+  </si>
+  <si>
+    <t>Desarmadores</t>
+  </si>
+  <si>
+    <t>Llaves</t>
+  </si>
+  <si>
+    <t>Martillos</t>
+  </si>
+  <si>
+    <t>Cinceles y punzones</t>
+  </si>
+  <si>
+    <t>Sierras manuales</t>
+  </si>
+  <si>
+    <t>Cuchillas y cutters</t>
+  </si>
+  <si>
+    <t>Juegos de herramientas</t>
+  </si>
+  <si>
+    <t>Winchas</t>
+  </si>
+  <si>
+    <t>Niveles</t>
+  </si>
+  <si>
+    <t>Escuadras</t>
+  </si>
+  <si>
+    <t>Tijeras de podar</t>
+  </si>
+  <si>
+    <t>Palas y picos</t>
+  </si>
+  <si>
+    <t>Rastrillos</t>
+  </si>
+  <si>
+    <t>Mangueras</t>
+  </si>
+  <si>
+    <t>Carretillas</t>
+  </si>
+  <si>
+    <t>Badilejos y planchas</t>
+  </si>
+  <si>
+    <t>Plomadas</t>
+  </si>
+  <si>
+    <t>Baldes</t>
+  </si>
+  <si>
+    <t>Llaves para tubo</t>
+  </si>
+  <si>
+    <t>Cortatubos</t>
+  </si>
+  <si>
+    <t>Cables</t>
+  </si>
+  <si>
+    <t>Interruptores y tomacorrientes</t>
+  </si>
+  <si>
+    <t>Cintas aislantes</t>
+  </si>
+  <si>
+    <t>Guantes</t>
+  </si>
+  <si>
+    <t>Lentes de seguridad</t>
+  </si>
+  <si>
+    <t>Respiradores y mascarillas</t>
+  </si>
+  <si>
+    <t>Calzado de seguridad</t>
+  </si>
+  <si>
+    <t>Chalecos reflectivos</t>
+  </si>
+  <si>
+    <t>Ropa de trabajo</t>
+  </si>
+  <si>
+    <t>Conos de seguridad</t>
+  </si>
+  <si>
+    <t>Barreras y mallas</t>
+  </si>
+  <si>
+    <t>Extintores</t>
+  </si>
+  <si>
+    <t>Botiquines</t>
+  </si>
+  <si>
+    <t>Discos de corte</t>
+  </si>
+  <si>
+    <t>Discos de desbaste</t>
+  </si>
+  <si>
+    <t>Brocas</t>
+  </si>
+  <si>
+    <t>Puntas y dados</t>
+  </si>
+  <si>
+    <t>Lijas</t>
+  </si>
+  <si>
+    <t>Hojas de sierra</t>
+  </si>
+  <si>
+    <t>Electrodos</t>
+  </si>
+  <si>
+    <t>Cajas de herramientas</t>
+  </si>
+  <si>
+    <t>Maletines</t>
+  </si>
+  <si>
+    <t>Organizadores</t>
+  </si>
+  <si>
+    <t>Protección colectiva</t>
+  </si>
+  <si>
+    <t>Subcategorías</t>
+  </si>
+  <si>
+    <t>Sierras eléctricas</t>
+  </si>
+  <si>
+    <t>Medidores láser</t>
+  </si>
+  <si>
+    <t>Teflón y selladores</t>
+  </si>
+  <si>
+    <t>Probadores y multímetros</t>
+  </si>
+  <si>
+    <t>Protección auditiva</t>
+  </si>
+  <si>
+    <t>Arneses y líneas de vida</t>
+  </si>
+  <si>
+    <t>Cintas de señalización</t>
+  </si>
+  <si>
+    <t>Señalética</t>
+  </si>
+  <si>
+    <t>3. Marca, Categoría, Subcategoría, Unidad, Garantía, Destacado y Activo se eligen de una lista desplegable.</t>
+  </si>
+  <si>
+    <t>CAS-B</t>
+  </si>
+  <si>
+    <t>Casco de seguridad tipo jockey con ajuste ratchet.</t>
+  </si>
+  <si>
+    <t>Material: polietileno de alta densidad; Ajuste: ratchet de 6 puntos; Color: blanco; Uso: construcción e industria</t>
+  </si>
+  <si>
+    <t>TRU-CAS-001.jpg</t>
+  </si>
+  <si>
+    <t>Distribuidora XYZ</t>
+  </si>
+  <si>
+    <t>Casco de seguridad tipo jockey fabricado en polietileno de alta densidad, liviano y resistente a impactos. Ideal para obras de construcción, talleres e industria.
+Su sistema de ajuste ratchet permite regularlo rápidamente a la medida de la cabeza, incluso con guantes puestos.
+- Suspensión de 6 puntos para mayor comodidad
+- Ranuras laterales para accesorios (orejeras o careta)
+- Banda de sudor reemplazable
+Recomendación: reemplaza el casco si recibe un golpe fuerte o presenta fisuras.</t>
   </si>
 </sst>
 </file>
@@ -504,7 +728,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -571,7 +795,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -877,42 +1108,42 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
@@ -920,7 +1151,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -958,7 +1189,7 @@
   <sheetData>
     <row r="1" spans="1:25" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -983,141 +1214,141 @@
       <c r="V1" s="29"/>
       <c r="W1" s="29"/>
       <c r="X1" s="29"/>
+      <c r="Y1" s="30"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
+      <c r="A2" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
+      <c r="S2" s="31"/>
+      <c r="T2" s="31"/>
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="30"/>
     </row>
     <row r="3" spans="1:25" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="20" t="s">
+      <c r="K3" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="20" t="s">
+      <c r="L3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="20" t="s">
+      <c r="M3" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="20" t="s">
+      <c r="N3" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="20" t="s">
+      <c r="O3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="Q3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="S3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="T3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="U3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="W3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="W3" s="3" t="s">
+      <c r="X3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="X3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>Descripción larga</t>
-        </is>
+      <c r="Y3" s="3" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="C4" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="19" t="s">
-        <v>45</v>
-      </c>
       <c r="I4" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J4" s="21">
         <v>150</v>
@@ -1151,56 +1382,52 @@
         <v>OK</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T4" s="26">
         <v>1.9</v>
       </c>
       <c r="U4" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="V4" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="V4" s="12" t="s">
-        <v>48</v>
-      </c>
       <c r="W4" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="X4" s="13"/>
-      <c r="Y4" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Taladro percutor de 650 W ideal para perforar concreto, ladrillo, madera y metal. Su función de percusión facilita el trabajo en superficies duras, y el giro reversible permite atornillar y destornillar con comodidad.
-Tiene mandril de 1/2" para brocas de distintos tamaños y velocidad variable de 0 a 3000 rpm para controlar cada perforación. Perfecto para instalaciones, remodelaciones y mantenimiento en casa, taller u obra.
-Recomendación: usa lentes de protección y guantes durante el trabajo.</t>
-        </is>
+      <c r="Y4" s="18" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="C5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="12" t="s">
+      <c r="F5" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="G5" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="19" t="s">
-        <v>55</v>
-      </c>
       <c r="I5" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J5" s="21">
         <v>110</v>
@@ -1232,56 +1459,52 @@
         <v>OK</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T5" s="26">
         <v>1.8</v>
       </c>
       <c r="U5" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="V5" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="V5" s="12" t="s">
-        <v>57</v>
-      </c>
       <c r="W5" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="X5" s="13"/>
-      <c r="Y5" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Amoladora angular de 750 W para cortar y desbastar metal, concreto, cerámica y piedra con discos de 4 1/2" (115 mm). Su motor de 11 000 rpm ofrece cortes rápidos y precisos.
-Cuenta con mango lateral para un mejor control y guarda de protección. Ideal para metalmecánica, construcción y mantenimiento.
-Recomendación: usa siempre lentes o careta de protección, guantes y el disco adecuado para cada material.</t>
-        </is>
+      <c r="Y5" s="18" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="C6" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="D6" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="F6" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="H6" s="19" t="s">
-        <v>64</v>
-      </c>
       <c r="I6" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J6" s="21">
         <v>14</v>
@@ -1313,67 +1536,105 @@
         <v>OK</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="T6" s="26">
         <v>0.35</v>
       </c>
       <c r="U6" s="27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="V6" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="W6" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="X6" s="13"/>
-      <c r="Y6" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Alicate universal de 8" fabricado en acero alto carbono, con cuerpo forjado y filos endurecidos para cortar, sujetar, doblar y torcer alambres y cables.
-Sus mangos ergonómicos de PVC bicolor brindan un agarre firme y cómodo durante el uso prolongado. Una herramienta básica para electricistas, mecánicos, técnicos y el hogar.
-Importante: el mango no está aislado; no lo uses en circuitos con corriente eléctrica.</t>
-        </is>
+      <c r="Y6" s="18" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="23" t="str">
+      <c r="A7" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="21">
+        <v>12</v>
+      </c>
+      <c r="K7" s="21">
+        <v>25</v>
+      </c>
+      <c r="L7" s="21">
+        <v>22</v>
+      </c>
+      <c r="M7" s="23">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="N7" s="23" t="str">
+        <v>22</v>
+      </c>
+      <c r="N7" s="23">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="O7" s="24" t="str">
+        <v>10</v>
+      </c>
+      <c r="O7" s="24">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="P7" s="12">
+        <v>40</v>
+      </c>
+      <c r="Q7" s="12">
+        <v>10</v>
+      </c>
       <c r="R7" s="25" t="str">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="S7" s="12"/>
-      <c r="T7" s="26"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="12"/>
-      <c r="W7" s="12"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="14"/>
+        <v>OK</v>
+      </c>
+      <c r="S7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="T7" s="26">
+        <v>0.4</v>
+      </c>
+      <c r="U7" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="V7" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="W7" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="X7" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="Y7" s="32" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="8" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
@@ -9038,7 +9299,7 @@
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
             <xm:f>Listas!$A$2:$A$20</xm:f>
@@ -9084,6 +9345,12 @@
           </x14:formula2>
           <xm:sqref>V4:W203</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Subcategoría" error="Esta subcategoría no está en la lista. Puedes dejarla así o agregarla en la hoja Listas (columna Subcategorías)." xr:uid="{00C130C2-9BF9-43CF-8B52-AAD5630B6443}">
+          <x14:formula1>
+            <xm:f>Listas!$F$2:$F$120</xm:f>
+          </x14:formula1>
+          <xm:sqref>E4:E203</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -9092,138 +9359,485 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="C3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="E3" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="D5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>82</v>
+      <c r="F6" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>85</v>
+      <c r="F7" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>87</v>
+      <c r="F8" s="6" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
-        <v>90</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F13" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F14" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F15" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F16" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F18" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F19" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F20" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F21" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F22" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F23" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F24" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F25" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="26" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F26" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F27" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="28" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F28" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F29" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F30" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="31" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F31" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="32" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F32" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F33" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="34" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F34" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="35" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F35" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="36" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F36" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F37" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F38" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="39" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F39" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="40" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F40" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F41" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F42" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F43" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="44" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F44" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="45" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F45" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="46" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F46" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="47" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F47" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="48" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F48" s="6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="49" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F49" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="50" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F50" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F51" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F52" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="53" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F53" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F54" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F55" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="56" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F56" s="6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="57" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F57" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="58" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F58" s="6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="59" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F59" s="6" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F60" s="6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="61" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F61" s="6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="62" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F62" s="6"/>
+    </row>
+    <row r="63" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F63" s="6"/>
+    </row>
+    <row r="64" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F64" s="6"/>
+    </row>
+    <row r="65" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F65" s="6"/>
+    </row>
+    <row r="66" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F66" s="6"/>
+    </row>
+    <row r="67" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F67" s="6"/>
+    </row>
+    <row r="68" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F68" s="6"/>
+    </row>
+    <row r="69" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F69" s="6"/>
+    </row>
+    <row r="70" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F70" s="6"/>
+    </row>
+    <row r="71" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F71" s="6"/>
+    </row>
+    <row r="72" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F72" s="6"/>
+    </row>
+    <row r="73" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F73" s="6"/>
+    </row>
+    <row r="74" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F74" s="6"/>
+    </row>
+    <row r="75" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F75" s="6"/>
+    </row>
+    <row r="76" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F76" s="6"/>
+    </row>
+    <row r="77" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F77" s="6"/>
+    </row>
+    <row r="78" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F78" s="6"/>
+    </row>
+    <row r="79" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F79" s="6"/>
+    </row>
+    <row r="80" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F80" s="6"/>
+    </row>
+    <row r="81" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F81" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9243,42 +9857,42 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B3" s="8">
         <f>COUNTA(Productos!A4:A203)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="8">
         <f>COUNTIF(Productos!W4:W203,"Sí")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B5" s="8">
         <f>COUNTIF(Productos!R4:R203,"Agotado")</f>
@@ -9290,16 +9904,16 @@
       </c>
       <c r="E5" s="9">
         <f>COUNTIF(Productos!C4:C203,D5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="9">
         <f>SUMIF(Productos!C4:C203,D5,Productos!P4:P203)</f>
-        <v>12</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B6" s="8">
         <f>COUNTIF(Productos!R4:R203,"Reponer")</f>
@@ -9320,11 +9934,11 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B7" s="10">
         <f>SUMPRODUCT(Productos!J4:J203,Productos!P4:P203)</f>
-        <v>3100</v>
+        <v>3580</v>
       </c>
       <c r="D7" s="9" t="str">
         <f>Listas!A4</f>
@@ -9341,11 +9955,11 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B8" s="10">
         <f>SUMPRODUCT(--(Productos!M4:M203&lt;&gt;""),Productos!P4:P203,N(+Productos!M4:M203))</f>
-        <v>4490</v>
+        <v>5370</v>
       </c>
       <c r="D8" s="9" t="str">
         <f>Listas!A5</f>
@@ -9362,11 +9976,11 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B9" s="11">
         <f>IFERROR(AVERAGE(Productos!O4:O203),0)</f>
-        <v>0.3451145272714658</v>
+        <v>0.37247225908996301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar kit Stanley FatMax V20 (STA-KIT-001)
Kit taladro percutor + atornillador de impacto brushless 18V V20, con foto.
Stanley agregado a la lista de marcas del catálogo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Productos_Herramientas.xlsx
+++ b/Catalogo_Productos_Herramientas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leo-n\Desktop\Claude Proyectos\1. Tienda Herramientas Online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458024BD-ED82-494C-AA55-E56EEA7FE0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0B1961-3AAD-414D-92E8-E9846BC06347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="182">
   <si>
     <t>CÓMO USAR ESTA PLANTILLA</t>
   </si>
@@ -600,6 +600,37 @@
 - Ranuras laterales para accesorios (orejeras o careta)
 - Banda de sudor reemplazable
 Recomendación: reemplaza el casco si recibe un golpe fuerte o presenta fisuras.</t>
+  </si>
+  <si>
+    <t>Stanley</t>
+  </si>
+  <si>
+    <t>STA-KIT-001</t>
+  </si>
+  <si>
+    <t>Kit taladro percutor + atornillador de impacto brushless 18V V20</t>
+  </si>
+  <si>
+    <t>SFMCK211D2T</t>
+  </si>
+  <si>
+    <t>Kit inalámbrico FatMax V20 con taladro percutor y atornillador de impacto sin carbones, 2 baterías y maletín.</t>
+  </si>
+  <si>
+    <t>Línea: Stanley FatMax V20 (18 V); Taladro percutor: motor brushless, torque máx. 80 Nm; Portabrocas: metálico de 13 mm (1/2"); Velocidades del taladro: 2 (0-500 / 0-2000 rpm); Percusión: 0-5950 / 0-25 500 ipm; Posiciones de torque: 15 + 2 (taladro y percusión); Atornillador de impacto: motor brushless, torque máx. 203 Nm; Porta puntas: hexagonal de 1/4"; Velocidades del atornillador: 3 (1400 / 2400 / 3200 rpm); Impactos por minuto: 4200 ipm; Incluye: 2 baterías Li-Ion 18 V de 2 Ah, cargador de 2 A y maletín Pro-Stack</t>
+  </si>
+  <si>
+    <t>STA-KIT-001.jpg</t>
+  </si>
+  <si>
+    <t>Kit inalámbrico Stanley FatMax V20 de 18 V que reúne dos herramientas esenciales: un taladro percutor y un atornillador de impacto, ambos con motor brushless (sin carbones), que entrega más potencia, mayor duración de la batería y menos mantenimiento.
+El taladro percutor ofrece hasta 80 Nm de torque, portabrocas metálico de 13 mm y dos velocidades para perforar concreto, ladrillo, madera y metal, o atornillar con precisión. El atornillador de impacto alcanza 203 Nm con tres velocidades, ideal para tornillos largos, pernos y fijaciones exigentes.
+- Motores brushless: más eficiencia y vida útil
+- Taladro con 15 + 2 posiciones de torque y función de percusión
+- Atornillador de impacto con 3 velocidades y porta puntas de 1/4"
+- Incluye 2 baterías Li-Ion 18 V de 2 Ah, cargador de 2 A y maletín Pro-Stack
+- Baterías compatibles con las demás herramientas de la línea V20
+Recomendación: usa lentes de protección y guantes; elige la velocidad baja para atornillar y la alta para perforar.</t>
   </si>
 </sst>
 </file>
@@ -611,7 +642,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;S/.&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -674,6 +705,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -728,7 +765,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -794,13 +831,16 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1188,62 +1228,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="31"/>
+      <c r="Y1" s="32"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
-      <c r="T2" s="31"/>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="30"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="33"/>
+      <c r="T2" s="33"/>
+      <c r="U2" s="33"/>
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+      <c r="Y2" s="32"/>
     </row>
     <row r="3" spans="1:25" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1559,7 +1599,7 @@
       <c r="A7" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="30" t="s">
         <v>107</v>
       </c>
       <c r="C7" s="12" t="s">
@@ -1632,48 +1672,88 @@
       <c r="X7" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="Y7" s="32" t="s">
+      <c r="Y7" s="29" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="23" t="str">
+      <c r="A8" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J8" s="21">
+        <v>550</v>
+      </c>
+      <c r="K8" s="21">
+        <v>720</v>
+      </c>
+      <c r="L8" s="21">
+        <v>700</v>
+      </c>
+      <c r="M8" s="23">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="N8" s="23" t="str">
+        <v>700</v>
+      </c>
+      <c r="N8" s="23">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="O8" s="24" t="str">
+        <v>150</v>
+      </c>
+      <c r="O8" s="24">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
+        <v>0.21428571428571427</v>
+      </c>
+      <c r="P8" s="12">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="12">
+        <v>5</v>
+      </c>
       <c r="R8" s="25" t="str">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="S8" s="12"/>
-      <c r="T8" s="26"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="12"/>
-      <c r="W8" s="12"/>
+        <v>OK</v>
+      </c>
+      <c r="S8" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="T8" s="26">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="U8" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="V8" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="W8" s="12" t="s">
+        <v>47</v>
+      </c>
       <c r="X8" s="13"/>
-      <c r="Y8" s="14"/>
+      <c r="Y8" s="14" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="9" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
@@ -1950,7 +2030,7 @@
     </row>
     <row r="16" spans="1:25" s="15" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
@@ -9448,7 +9528,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>76</v>
+        <v>174</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>77</v>
@@ -9464,6 +9544,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
       <c r="B6" s="6" t="s">
         <v>79</v>
       </c>
@@ -9866,7 +9949,7 @@
       </c>
       <c r="B3" s="8">
         <f>COUNTA(Productos!A4:A203)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>92</v>
@@ -9878,7 +9961,7 @@
       </c>
       <c r="B4" s="8">
         <f>COUNTIF(Productos!W4:W203,"Sí")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>15</v>
@@ -9938,7 +10021,7 @@
       </c>
       <c r="B7" s="10">
         <f>SUMPRODUCT(Productos!J4:J203,Productos!P4:P203)</f>
-        <v>3580</v>
+        <v>9080</v>
       </c>
       <c r="D7" s="9" t="str">
         <f>Listas!A4</f>
@@ -9959,19 +10042,19 @@
       </c>
       <c r="B8" s="10">
         <f>SUMPRODUCT(--(Productos!M4:M203&lt;&gt;""),Productos!P4:P203,N(+Productos!M4:M203))</f>
-        <v>5370</v>
+        <v>12370</v>
       </c>
       <c r="D8" s="9" t="str">
         <f>Listas!A5</f>
-        <v>Otra</v>
+        <v>Stanley</v>
       </c>
       <c r="E8" s="9">
         <f>COUNTIF(Productos!C4:C203,D8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="9">
         <f>SUMIF(Productos!C4:C203,D8,Productos!P4:P203)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -9980,7 +10063,7 @@
       </c>
       <c r="B9" s="11">
         <f>IFERROR(AVERAGE(Productos!O4:O203),0)</f>
-        <v>0.37247225908996301</v>
+        <v>0.34083495012911325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>